<commit_message>
docs(carga-masiva): los pasos para recorrer el flujo a mano
El README suma la seccion "Como recorrer el flujo a mano": que marcar en
el paso 2 y que mirar en el paso 3, de arriba abajo, con el archivo
guiado. Hasta ahora eso vivia en la conversacion y se perdia.

Se anotan tambien los dos cambios de la hoja de compatibilidades: que se
edita y se le agregan autos, y que la clave de una correccion apunta a un
auto y no a una fila.

El archivo guiado suma una fila con el codigo repetido, que es la otra
forma de traer varias compatibilidades —la que ofrece el interruptor de
juntar filas repetidas—. Con eso el recorrido pasa por los dos caminos y
la hoja del Excel sale con tres filas en vez de dos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pruebas-crudas/12-prueba-guiada.xlsx
+++ b/pruebas-crudas/12-prueba-guiada.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -608,30 +608,53 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>PF-201</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Pastilla freno delantera</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Bosch</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Frenos</v>
+      </c>
+      <c r="E10">
+        <v>24990</v>
+      </c>
+      <c r="F10">
+        <v>12</v>
+      </c>
+      <c r="G10" t="str">
+        <v>NISSAN V16 1995-2008</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v/>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>SUBTOTAL</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C11" t="str">
         <v/>
       </c>
-      <c r="D10" t="str">
+      <c r="D11" t="str">
         <v/>
       </c>
-      <c r="E10">
+      <c r="E11">
         <v>237930</v>
       </c>
-      <c r="F10">
+      <c r="F11">
         <v>68</v>
       </c>
-      <c r="G10" t="str">
+      <c r="G11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>